<commit_message>
A9 settled by Brennan 5405-24-24 / -32-32 (tap drill -24 1.72, -32 2.20); user decisions recorded; stage now 8 new configurations
Q-CODE62-CAT = Brennan table 3300-62; FS2408 as Brennan builds it; 6801-L / -LL folded as 2501-L.
Checks over the 39 regenerated roots clean.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PJcT2926CUEincCxCV1ZSx
</commit_message>
<xml_diff>
--- a/tools/_out/brennancad_20261021/regen/stage/straight/DesignTable_5000_SW2.xlsx
+++ b/tools/_out/brennancad_20261021/regen/stage/straight/DesignTable_5000_SW2.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AB23"/>
+  <dimension ref="A1:AB24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2384,17 +2384,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>5000-24-24</t>
+          <t>5000-24-20</t>
         </is>
       </c>
       <c r="B20" t="n">
         <v>1.93</v>
       </c>
       <c r="C20" t="n">
-        <v>1.37409</v>
+        <v>1.37121</v>
       </c>
       <c r="D20" t="n">
-        <v>2.38</v>
+        <v>2.375</v>
       </c>
       <c r="E20" t="n">
         <v>1.72</v>
@@ -2418,13 +2418,13 @@
         <v>0.9296</v>
       </c>
       <c r="L20" t="n">
-        <v>1.72</v>
+        <v>1.48</v>
       </c>
       <c r="M20" t="n">
         <v>1.16</v>
       </c>
       <c r="N20" t="n">
-        <v>1.72</v>
+        <v>1.48</v>
       </c>
       <c r="O20" t="n">
         <v>0.965</v>
@@ -2433,22 +2433,22 @@
         <v>0.08699999999999999</v>
       </c>
       <c r="Q20" t="n">
-        <v>0.86</v>
+        <v>0.74</v>
       </c>
       <c r="R20" t="n">
-        <v>0.9296</v>
+        <v>0.8096</v>
       </c>
       <c r="S20" t="n">
         <v>1.93</v>
       </c>
       <c r="T20" t="inlineStr">
         <is>
-          <t>5000-24-24</t>
+          <t>5000-24-20</t>
         </is>
       </c>
       <c r="U20" t="inlineStr">
         <is>
-          <t>Hexagon Pipe Coupling, 1 1/2-11 1/2 NPTF (female) x 1 1/2-11 1/2 NPTF (female)</t>
+          <t>Hexagon Pipe Coupling, 1 1/2-11 1/2 NPTF (female) x 1 1/4-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="V20" t="inlineStr">
@@ -2463,7 +2463,7 @@
       </c>
       <c r="X20" t="inlineStr">
         <is>
-          <t>1 1/2-11 1/2 NPTF (female)</t>
+          <t>1 1/4-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="Y20" t="inlineStr">
@@ -2473,50 +2473,55 @@
       </c>
       <c r="Z20" t="inlineStr">
         <is>
-          <t>Air-Way s82 only (double-pass 19 rows); female NPTF per ANSI B1.20.3 | MODEL: female NPTF drill depth = MS51503 P1 max per pipe dash (2405 table); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); the two drill holes are cut to max(P1, L/2+0.005) so the coupling is through (ASSUMPTION); each helical thread is cut to min(P1, L/2) (ASSUMPTION - for -08 this equals the Brennan thread depth 0.75); hex spans the full length</t>
+          <t>[A1/A9 TAPDRILL 2026-10-21: TAPDRILL2@BORE] [A1/A9 TAPDRILL 2026-10-21: TAPDRILL1@BORE] [BRENNAN-CAD 2026-10-21: CHEX@HEX, L@DRIVE, THDMAJ_A1@DRIVE, THDMAJ_A2@DRIVE] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING | MODEL: female NPTF drill depth = MS51503 P1 max per pipe dash (2405 table); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); the two drill holes are cut to max(P1, L/2+0.005) so the coupling is through (ASSUMPTION); each helical thread is cut to min(P1, L/2) (ASSUMPTION - for -08 this equals the Brennan thread depth 0.75); hex spans the full length</t>
+        </is>
+      </c>
+      <c r="AA20" t="inlineStr">
+        <is>
+          <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | Brennan CAD record 5000-24-20 (PARTcommunity / CADENAS, CHEX@HEX=C, L@DRIVE=L, THDMAJ_A1@DRIVE=A1THD, THDMAJ_A2@DRIVE=A2THD; user 2026-10-21 "yes you can use them following my rule") | TAPDRILL1@BORE = Air-Way per-size tap drill -24 1.72 (A1, A9: Brennan 5405-24-24 / -32-32 STEPs 1.734 / 2.218 -&gt; nearest Air-Way 1.72 / 2.20) | TAPDRILL2@BORE = Air-Way per-size tap drill -20 1.48 (A1)</t>
         </is>
       </c>
       <c r="AB20" t="inlineStr">
         <is>
-          <t>5000-24-24</t>
+          <t>5000-24-20</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>5000-32-24</t>
+          <t>5000-24-24</t>
         </is>
       </c>
       <c r="B21" t="n">
-        <v>1.96</v>
+        <v>1.93</v>
       </c>
       <c r="C21" t="n">
-        <v>1.66277</v>
+        <v>1.37409</v>
       </c>
       <c r="D21" t="n">
-        <v>2.88</v>
+        <v>2.38</v>
       </c>
       <c r="E21" t="n">
-        <v>2.2</v>
+        <v>1.72</v>
       </c>
       <c r="F21" t="n">
-        <v>1.18</v>
+        <v>1.16</v>
       </c>
       <c r="G21" t="n">
-        <v>2.2</v>
+        <v>1.72</v>
       </c>
       <c r="H21" t="n">
-        <v>0.98</v>
+        <v>0.965</v>
       </c>
       <c r="I21" t="n">
         <v>0.08699999999999999</v>
       </c>
       <c r="J21" t="n">
-        <v>1.1</v>
+        <v>0.86</v>
       </c>
       <c r="K21" t="n">
-        <v>1.1696</v>
+        <v>0.9296</v>
       </c>
       <c r="L21" t="n">
         <v>1.72</v>
@@ -2528,7 +2533,7 @@
         <v>1.72</v>
       </c>
       <c r="O21" t="n">
-        <v>0.98</v>
+        <v>0.965</v>
       </c>
       <c r="P21" t="n">
         <v>0.08699999999999999</v>
@@ -2540,16 +2545,16 @@
         <v>0.9296</v>
       </c>
       <c r="S21" t="n">
-        <v>1.96</v>
+        <v>1.93</v>
       </c>
       <c r="T21" t="inlineStr">
         <is>
-          <t>5000-32-24</t>
+          <t>5000-24-24</t>
         </is>
       </c>
       <c r="U21" t="inlineStr">
         <is>
-          <t>Hexagon Pipe Coupling, 2-11 1/2 NPTF (female) x 1 1/2-11 1/2 NPTF (female)</t>
+          <t>Hexagon Pipe Coupling, 1 1/2-11 1/2 NPTF (female) x 1 1/2-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="V21" t="inlineStr">
@@ -2559,7 +2564,7 @@
       </c>
       <c r="W21" t="inlineStr">
         <is>
-          <t>2-11 1/2 NPTF (female)</t>
+          <t>1 1/2-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="X21" t="inlineStr">
@@ -2577,21 +2582,16 @@
           <t>Air-Way s82 only (double-pass 19 rows); female NPTF per ANSI B1.20.3 | MODEL: female NPTF drill depth = MS51503 P1 max per pipe dash (2405 table); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); the two drill holes are cut to max(P1, L/2+0.005) so the coupling is through (ASSUMPTION); each helical thread is cut to min(P1, L/2) (ASSUMPTION - for -08 this equals the Brennan thread depth 0.75); hex spans the full length</t>
         </is>
       </c>
-      <c r="AA21" t="inlineStr">
-        <is>
-          <t>TapDrill(1) 2.20 vs 32-32 2.19 for the same 2-11 1/2 thread - as-printed</t>
-        </is>
-      </c>
       <c r="AB21" t="inlineStr">
         <is>
-          <t>5000-32-24</t>
+          <t>5000-24-24</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>5000-32-32</t>
+          <t>5000-32-24</t>
         </is>
       </c>
       <c r="B22" t="n">
@@ -2604,13 +2604,13 @@
         <v>2.88</v>
       </c>
       <c r="E22" t="n">
-        <v>2.19</v>
+        <v>2.2</v>
       </c>
       <c r="F22" t="n">
         <v>1.18</v>
       </c>
       <c r="G22" t="n">
-        <v>2.19</v>
+        <v>2.2</v>
       </c>
       <c r="H22" t="n">
         <v>0.98</v>
@@ -2619,19 +2619,19 @@
         <v>0.08699999999999999</v>
       </c>
       <c r="J22" t="n">
-        <v>1.095</v>
+        <v>1.1</v>
       </c>
       <c r="K22" t="n">
-        <v>1.1646</v>
+        <v>1.1696</v>
       </c>
       <c r="L22" t="n">
-        <v>2.19</v>
+        <v>1.72</v>
       </c>
       <c r="M22" t="n">
-        <v>1.18</v>
+        <v>1.16</v>
       </c>
       <c r="N22" t="n">
-        <v>2.19</v>
+        <v>1.72</v>
       </c>
       <c r="O22" t="n">
         <v>0.98</v>
@@ -2640,22 +2640,22 @@
         <v>0.08699999999999999</v>
       </c>
       <c r="Q22" t="n">
-        <v>1.095</v>
+        <v>0.86</v>
       </c>
       <c r="R22" t="n">
-        <v>1.1646</v>
+        <v>0.9296</v>
       </c>
       <c r="S22" t="n">
         <v>1.96</v>
       </c>
       <c r="T22" t="inlineStr">
         <is>
-          <t>5000-32-32</t>
+          <t>5000-32-24</t>
         </is>
       </c>
       <c r="U22" t="inlineStr">
         <is>
-          <t>Hexagon Pipe Coupling, 2-11 1/2 NPTF (female) x 2-11 1/2 NPTF (female)</t>
+          <t>Hexagon Pipe Coupling, 2-11 1/2 NPTF (female) x 1 1/2-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="V22" t="inlineStr">
@@ -2670,7 +2670,7 @@
       </c>
       <c r="X22" t="inlineStr">
         <is>
-          <t>2-11 1/2 NPTF (female)</t>
+          <t>1 1/2-11 1/2 NPTF (female)</t>
         </is>
       </c>
       <c r="Y22" t="inlineStr">
@@ -2683,113 +2683,219 @@
           <t>Air-Way s82 only (double-pass 19 rows); female NPTF per ANSI B1.20.3 | MODEL: female NPTF drill depth = MS51503 P1 max per pipe dash (2405 table); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); the two drill holes are cut to max(P1, L/2+0.005) so the coupling is through (ASSUMPTION); each helical thread is cut to min(P1, L/2) (ASSUMPTION - for -08 this equals the Brennan thread depth 0.75); hex spans the full length</t>
         </is>
       </c>
+      <c r="AA22" t="inlineStr">
+        <is>
+          <t>TapDrill(1) 2.20 vs 32-32 2.19 for the same 2-11 1/2 thread - as-printed</t>
+        </is>
+      </c>
       <c r="AB22" t="inlineStr">
         <is>
-          <t>5000-32-32</t>
+          <t>5000-32-24</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>5000-32-32</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="C23" t="n">
+        <v>1.66277</v>
+      </c>
+      <c r="D23" t="n">
+        <v>2.88</v>
+      </c>
+      <c r="E23" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="F23" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="G23" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="H23" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="I23" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="J23" t="n">
+        <v>1.095</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1.1646</v>
+      </c>
+      <c r="L23" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="M23" t="n">
+        <v>1.18</v>
+      </c>
+      <c r="N23" t="n">
+        <v>2.19</v>
+      </c>
+      <c r="O23" t="n">
+        <v>0.98</v>
+      </c>
+      <c r="P23" t="n">
+        <v>0.08699999999999999</v>
+      </c>
+      <c r="Q23" t="n">
+        <v>1.095</v>
+      </c>
+      <c r="R23" t="n">
+        <v>1.1646</v>
+      </c>
+      <c r="S23" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="T23" t="inlineStr">
+        <is>
+          <t>5000-32-32</t>
+        </is>
+      </c>
+      <c r="U23" t="inlineStr">
+        <is>
+          <t>Hexagon Pipe Coupling, 2-11 1/2 NPTF (female) x 2-11 1/2 NPTF (female)</t>
+        </is>
+      </c>
+      <c r="V23" t="inlineStr">
+        <is>
+          <t>5000</t>
+        </is>
+      </c>
+      <c r="W23" t="inlineStr">
+        <is>
+          <t>2-11 1/2 NPTF (female)</t>
+        </is>
+      </c>
+      <c r="X23" t="inlineStr">
+        <is>
+          <t>2-11 1/2 NPTF (female)</t>
+        </is>
+      </c>
+      <c r="Y23" t="inlineStr">
+        <is>
+          <t>ASSUMED</t>
+        </is>
+      </c>
+      <c r="Z23" t="inlineStr">
+        <is>
+          <t>Air-Way s82 only (double-pass 19 rows); female NPTF per ANSI B1.20.3 | MODEL: female NPTF drill depth = MS51503 P1 max per pipe dash (2405 table); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); the two drill holes are cut to max(P1, L/2+0.005) so the coupling is through (ASSUMPTION); each helical thread is cut to min(P1, L/2) (ASSUMPTION - for -08 this equals the Brennan thread depth 0.75); hex spans the full length</t>
+        </is>
+      </c>
+      <c r="AB23" t="inlineStr">
+        <is>
+          <t>5000-32-32</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>5000-40-40</t>
         </is>
       </c>
-      <c r="B23" t="n">
+      <c r="B24" t="n">
         <v>2.67</v>
       </c>
-      <c r="C23" t="n">
+      <c r="C24" t="n">
         <v>2.02073</v>
       </c>
-      <c r="D23" t="n">
+      <c r="D24" t="n">
         <v>3.5</v>
       </c>
-      <c r="E23" t="n">
+      <c r="E24" t="n">
         <v>2.729</v>
       </c>
-      <c r="F23" t="n">
+      <c r="F24" t="n">
         <v>1.34</v>
       </c>
-      <c r="G23" t="n">
+      <c r="G24" t="n">
         <v>2.729</v>
       </c>
-      <c r="H23" t="n">
+      <c r="H24" t="n">
         <v>1.0443</v>
       </c>
-      <c r="I23" t="n">
+      <c r="I24" t="n">
         <v>0.125</v>
       </c>
-      <c r="J23" t="n">
+      <c r="J24" t="n">
         <v>1.3645</v>
       </c>
-      <c r="K23" t="n">
+      <c r="K24" t="n">
         <v>1.4645</v>
       </c>
-      <c r="L23" t="n">
+      <c r="L24" t="n">
         <v>2.729</v>
       </c>
-      <c r="M23" t="n">
+      <c r="M24" t="n">
         <v>1.34</v>
       </c>
-      <c r="N23" t="n">
+      <c r="N24" t="n">
         <v>2.729</v>
       </c>
-      <c r="O23" t="n">
+      <c r="O24" t="n">
         <v>1.0443</v>
       </c>
-      <c r="P23" t="n">
+      <c r="P24" t="n">
         <v>0.125</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="Q24" t="n">
         <v>1.3645</v>
       </c>
-      <c r="R23" t="n">
+      <c r="R24" t="n">
         <v>1.4645</v>
       </c>
-      <c r="S23" t="n">
+      <c r="S24" t="n">
         <v>2.67</v>
       </c>
-      <c r="T23" t="inlineStr">
+      <c r="T24" t="inlineStr">
         <is>
           <t>5000-40-40</t>
         </is>
       </c>
-      <c r="U23" t="inlineStr">
+      <c r="U24" t="inlineStr">
         <is>
           <t>Hexagon Pipe Coupling, 2 1/2-8 NPTF (female) x 2 1/2-8 NPTF (female)</t>
         </is>
       </c>
-      <c r="V23" t="inlineStr">
+      <c r="V24" t="inlineStr">
         <is>
           <t>5000</t>
         </is>
       </c>
-      <c r="W23" t="inlineStr">
+      <c r="W24" t="inlineStr">
         <is>
           <t>2 1/2-8 NPTF (female)</t>
         </is>
       </c>
-      <c r="X23" t="inlineStr">
+      <c r="X24" t="inlineStr">
         <is>
           <t>2 1/2-8 NPTF (female)</t>
         </is>
       </c>
-      <c r="Y23" t="inlineStr">
+      <c r="Y24" t="inlineStr">
         <is>
           <t>ASSUMED</t>
         </is>
       </c>
-      <c r="Z23" t="inlineStr">
+      <c r="Z24" t="inlineStr">
         <is>
           <t>[BRENNAN-ONLY 2026-10-18] OMi catalog SKU (omindustrial.com collections feed (cs-adapters, carbon-steel-flange-adapters-accessories, carbon-steel-braze-beaded-hose; products.json limit=50, single pass 2026-09-23)); NO Air-Way row for this size -&gt; dimensions MISSING -&gt; 2026-10-18 Brennan allowed (user: "yes use brennan but still differentiate"); sources per cell in CHANGES.csv | MODEL: female NPTF drill depth = MS51503 P1 max per pipe dash (2405 table); Brennan 5405-08-08 STEP (2026-09-23) confirms 1/2 NPTF port drill depth 0.900 = MS51503 P1 max (VERIFIED for -08 only; thread taper depth in that STEP is 0.750, tap drill dia 0.718, drill point 120 deg); the two drill holes are cut to max(P1, L/2+0.005) so the coupling is through (ASSUMPTION); each helical thread is cut to min(P1, L/2) (ASSUMPTION - for -08 this equals the Brennan thread depth 0.75); hex spans the full length; -40 PIPE END (2-1/2-8 NPTF) IS BRENNAN-MEASURED, NOT ASME B1.20.1 (user 2026-10-02: Brennan-measured threads accepted for -40): male end - pitch dia at the tip E0 2.71954 = the Brennan blank cone 2.7769 (5404-40-40 / 5406-40-32 / 2501-40-40-FG STEPs) - 0.4589 P (the Brennan blank sits 0.4585-0.4595 P above ASME E0 at all 8 library sizes -04..-32, ASSUMED to hold at -40), crest E0 + 0.8P, taper 1.7899deg, thread length L2 1.1374 from D = E0 + 0.8P + (L2 - 2P)/16 with pipe OD D 2.875 (Brennan collar), end length 1.515 (measured on all four Brennan -40 male ends); female port - tap drill 2.729 and thread depth 1.0443 = the Brennan 5000-40-40 tapered port (no separate drill: the 2.729 bore runs through); 8 threads per inch = Brennan TFA catalog callout 2-1/2-8; single manufacturer, ASSUMED</t>
         </is>
       </c>
-      <c r="AA23" t="inlineStr">
+      <c r="AA24" t="inlineStr">
         <is>
           <t>BUILD-MISSING: part exists in OMi catalog but the Air-Way page has no row; needs a second dimensional source | 2026-10-18 Brennan = yes (wave 2 straight, staged, not shipped): L / hex from the Brennan TFA catalog p10 alone; -40 pipe ends not in the end library</t>
         </is>
       </c>
-      <c r="AB23" t="inlineStr">
+      <c r="AB24" t="inlineStr">
         <is>
           <t>5000-40-40</t>
         </is>

</xml_diff>